<commit_message>
feat(auth): implementar autenticacion obligatoria, autoregistro de stakeholders y exportacion nativa en Excel (.xlsx)
</commit_message>
<xml_diff>
--- a/BASE/SERIALES.xlsx
+++ b/BASE/SERIALES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Palmaseca\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity\Projects\Control Mod\BASE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5834EA90-0A2A-4A38-972E-D34C2A7710BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1586CB61-E3D1-41F6-91E2-563FBB68E9A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0D82A942-C1A7-4E1B-8E9A-7178D61A88B1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0D82A942-C1A7-4E1B-8E9A-7178D61A88B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -88,12 +85,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -108,11 +111,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -131,9 +132,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -171,7 +172,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -277,7 +278,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -419,7 +420,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -428,9 +429,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D076EE1-A6D6-45BA-A8C1-F723AB856B0F}">
   <dimension ref="A1:C47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +442,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -452,7 +453,7 @@
         <v>30778700</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -463,7 +464,7 @@
         <v>30778693</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -474,7 +475,7 @@
         <v>30778692</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -485,18 +486,18 @@
         <v>30778690</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6">
         <v>5</v>
       </c>
       <c r="C6">
         <v>30778687</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -507,7 +508,7 @@
         <v>30778681</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -518,7 +519,7 @@
         <v>30778697</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -529,7 +530,7 @@
         <v>30778673</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -540,7 +541,7 @@
         <v>30778672</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -551,7 +552,7 @@
         <v>30778670</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -562,7 +563,7 @@
         <v>30778661</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -573,7 +574,7 @@
         <v>30773509</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -584,7 +585,7 @@
         <v>30778688</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -595,7 +596,7 @@
         <v>30777967</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -606,29 +607,29 @@
         <v>30777962</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>5</v>
       </c>
       <c r="B17">
         <v>4</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17">
         <v>30777951</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>5</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="1">
         <v>30773512</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -639,7 +640,7 @@
         <v>30763827</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -650,7 +651,7 @@
         <v>30778680</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -661,18 +662,18 @@
         <v>30778679</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>6</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <v>30778677</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -683,259 +684,255 @@
         <v>30778676</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="2">
-        <v>5</v>
-      </c>
-      <c r="C24" s="3">
+      <c r="B24">
+        <v>5</v>
+      </c>
+      <c r="C24">
         <v>30773498</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B25">
         <v>1</v>
       </c>
-      <c r="C25" s="3">
+      <c r="C25">
         <v>30777965</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>7</v>
       </c>
-      <c r="B26" s="3">
-        <v>6</v>
-      </c>
-      <c r="C26" s="3">
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="C26">
         <v>30778699</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="3">
-        <v>4</v>
-      </c>
-      <c r="C27" s="3">
+      <c r="B27">
+        <v>4</v>
+      </c>
+      <c r="C27">
         <v>30778689</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28">
         <v>2</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28">
         <v>30778686</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29">
         <v>1</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29">
         <v>30777977</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="3">
-        <v>3</v>
-      </c>
-      <c r="C30" s="3">
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
         <v>30302105</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="3">
-        <v>5</v>
-      </c>
-      <c r="C31" s="2"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32">
         <v>2</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32">
         <v>30778703</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>8</v>
       </c>
-      <c r="B33" s="2">
-        <v>6</v>
-      </c>
-      <c r="C33" s="3">
+      <c r="B33">
+        <v>6</v>
+      </c>
+      <c r="C33">
         <v>30778682</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>8</v>
       </c>
-      <c r="B34" s="2">
-        <v>5</v>
-      </c>
-      <c r="C34" s="3">
+      <c r="B34">
+        <v>5</v>
+      </c>
+      <c r="C34">
         <v>30777976</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="3">
-        <v>4</v>
-      </c>
-      <c r="C35" s="3">
+      <c r="B35">
+        <v>4</v>
+      </c>
+      <c r="C35">
         <v>30777972</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>8</v>
       </c>
-      <c r="B36" s="3">
+      <c r="B36">
         <v>1</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36">
         <v>30777955</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="3">
-        <v>3</v>
-      </c>
-      <c r="C37" s="3">
+      <c r="B37">
+        <v>3</v>
+      </c>
+      <c r="C37">
         <v>30773510</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="3">
-        <v>5</v>
-      </c>
-      <c r="C38" s="3">
+      <c r="B38">
+        <v>5</v>
+      </c>
+      <c r="C38">
         <v>30778684</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="3">
-        <v>6</v>
-      </c>
-      <c r="C39" s="3">
+      <c r="B39">
+        <v>6</v>
+      </c>
+      <c r="C39">
         <v>30778683</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>9</v>
       </c>
-      <c r="B40" s="3">
+      <c r="B40">
         <v>1</v>
       </c>
-      <c r="C40" s="3">
+      <c r="C40">
         <v>30778678</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>9</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41">
         <v>2</v>
       </c>
-      <c r="C41" s="3"/>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="2">
-        <v>4</v>
-      </c>
-      <c r="C42" s="2"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>9</v>
       </c>
-      <c r="B43" s="3">
-        <v>3</v>
-      </c>
-      <c r="C43" s="2"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>10</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44">
         <v>2</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44">
         <v>30778701</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>10</v>
       </c>
-      <c r="B45" s="3">
-        <v>3</v>
-      </c>
-      <c r="C45" s="3">
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45">
         <v>30778691</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>10</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B46">
         <v>1</v>
       </c>
-      <c r="C46" s="2">
+      <c r="C46">
         <v>30778685</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>10</v>
       </c>
-      <c r="B47" s="2">
-        <v>4</v>
-      </c>
-      <c r="C47" s="2">
+      <c r="B47">
+        <v>4</v>
+      </c>
+      <c r="C47">
         <v>30777969</v>
       </c>
     </row>

</xml_diff>